<commit_message>
refactor(gamecore): harden runtime ownership and validation gates
- move owned ContextSteering2D code into ProjectPlugins and update references
- formalize runtime owner boundaries for resources, persistence, UI, quests, audio, commands, maps, and equipment presentation
- add focused static gate scripts and project decision records for the refactor
- update equipment animation/resource workflow assets, validators, scenes, and generated data
- strengthen save/reference handling to skip or reject unresolved registry assets instead of writing empty GUIDs
</commit_message>
<xml_diff>
--- a/EX_GAS_Config/ProjectConfigTable/exgas_config/Datas/#exgas.abilityGameCore.xlsx
+++ b/EX_GAS_Config/ProjectConfigTable/exgas_config/Datas/#exgas.abilityGameCore.xlsx
@@ -573,22 +573,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GameCore ability prefab GUID</t>
+          <t>GameCore PrefabReference database GUID</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>GameCore ability prefab runtime path/address</t>
+          <t>Optional ResourceSystem/Addressables runtime address; empty when PrefabGuid resolves through DatabaseRegistry</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>GameCore ability icon GUID</t>
+          <t>GameCore SpriteReference database GUID</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>GameCore ability icon runtime path/address</t>
+          <t>Optional ResourceSystem/Addressables runtime address; empty when IconGuid resolves through DatabaseRegistry</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -638,24 +638,16 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>24d29f17c2627fc4c89e281895e4aa89</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Assets/Prefabs/Abilities/Melee/测试-基础攻击.prefab</t>
-        </is>
-      </c>
+          <t>5b38e7a9c3224e3dbaa98c2b0dd07e05</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1c9b84d978891c24288defb67855d5f3</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Assets/Art/KrishnaPalacio/MINIFANTASY - Dungeon/Sprites/Animations/Human/HumanBaseAttack.png</t>
-        </is>
-      </c>
+          <t>eff924477cc645b79f2e586fbbfc7a50</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
         <v>1</v>
       </c>
@@ -687,14 +679,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>24d29f17c2627fc4c89e281895e4aa89</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Assets/Prefabs/Abilities/Melee/测试-基础攻击.prefab</t>
-        </is>
-      </c>
+          <t>5b38e7a9c3224e3dbaa98c2b0dd07e05</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
         <v>1</v>
       </c>
@@ -726,24 +716,16 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>24d29f17c2627fc4c89e281895e4aa89</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Assets/Prefabs/Abilities/Melee/测试-基础攻击.prefab</t>
-        </is>
-      </c>
+          <t>5b38e7a9c3224e3dbaa98c2b0dd07e05</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0b5262a6696fdd4479d0e186f7021230</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Assets/Art/KrishnaPalacio/MINIFANTASY - Dungeon/Sprites/Animations/Human/HumanBaseChargedAttack.png</t>
-        </is>
-      </c>
+          <t>a146817efeef4e999987241c5ccb6d5b</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
         <v>1</v>
       </c>
@@ -775,14 +757,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>a146750504c64be4a948e93b1a20e117</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Assets/Prefabs/Abilities/World/喷火.prefab</t>
-        </is>
-      </c>
+          <t>19f7e6400fc1490f894f4419c1d29ca9</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
         <v>1</v>
       </c>

</xml_diff>